<commit_message>
Cập nhật file mẫu nhập Excel: thêm cột Chuyên án + Số đầu 4X
- sample_data/mau_ma_lieu.xlsx: đổi sang 5 cột
  (Chuyên án | Tên mã liệu | Số đầu 4X | Số đầu 8X | Số đầu 16X),
  dữ liệu mẫu gom theo chuyên án (A: ABC/BCD, B: DEF/GHI, C: XYZ).
- README: cập nhật mục "nhập mã liệu từ Excel" và lưu trình cho khớp
  định dạng mới (Chuyên án → Mã liệu → Loại đầu 4X/8X/16X).

(Phần code nhận diện cột Chuyên án trong material_import đã có từ trước;
lần này bổ sung file mẫu và tài liệu cho đồng bộ.)

https://claude.ai/code/session_01CnTCFSkFu21tLp2fDSS1Zw
</commit_message>
<xml_diff>
--- a/mes_uploader_app/sample_data/mau_ma_lieu.xlsx
+++ b/mes_uploader_app/sample_data/mau_ma_lieu.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,26 +417,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Chuyên án</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Tên mã liệu</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Số đầu 4X</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Số đầu 8X</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Số đầu 16X</t>
         </is>
@@ -441,39 +457,105 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Chuyên án A</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
         <v>2</v>
       </c>
-      <c r="C2" t="n">
+      <c r="E2" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Chuyên án A</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>BCD</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
         <v>4</v>
       </c>
-      <c r="C3" t="n">
+      <c r="E3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Chuyên án B</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Chuyên án B</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>GHI</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Chuyên án C</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>XYZ</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="n">
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>